<commit_message>
feat: add ART cascade analysis and HTS reconciliation analysis components
- Implemented ArtCascadeAnalysis.vue for visualizing ART cascade data, including cohort outcomes, retention trends, and VL coverage.
- Added functionality for downloading charts and CSV data for ART cascade analysis.
- Created HtsReconciliationAnalysis.vue to compare HTS register against other evidence sources, highlighting gaps in data.
- Included download options for reconciliation records and charts in various formats.
</commit_message>
<xml_diff>
--- a/data/20260905_AHP_ Indicators_kpq.xlsx
+++ b/data/20260905_AHP_ Indicators_kpq.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="393">
   <si>
     <t>Indicator No.</t>
   </si>
@@ -1216,6 +1216,9 @@
   </si>
   <si>
     <t>STI-S (sti_access)</t>
+  </si>
+  <si>
+    <t>LD-2 (ld_postnatal_care)</t>
   </si>
 </sst>
 </file>
@@ -2770,7 +2773,9 @@
       <c r="K26" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="L26" s="3"/>
+      <c r="L26" s="3" t="s">
+        <v>392</v>
+      </c>
       <c r="M26" s="3" t="s">
         <v>321</v>
       </c>

</xml_diff>

<commit_message>
feat: update ART retention and LTFU indicators to align with new client-supplied methodology
</commit_message>
<xml_diff>
--- a/data/20260905_AHP_ Indicators_kpq.xlsx
+++ b/data/20260905_AHP_ Indicators_kpq.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="394">
   <si>
     <t>Indicator No.</t>
   </si>
@@ -570,9 +570,6 @@
     <t>Transfer Out</t>
   </si>
   <si>
-    <t>(Number alive and on ART at 12 months ÷ Number enrolled on ART 12 months earlier) × 100</t>
-  </si>
-  <si>
     <t>HTS</t>
   </si>
   <si>
@@ -1219,6 +1216,12 @@
   </si>
   <si>
     <t>LD-2 (ld_postnatal_care)</t>
+  </si>
+  <si>
+    <t>art</t>
+  </si>
+  <si>
+    <t>artr_registration_date,art_review_date,art_registration_date,art_visit_number, art_final_outcome</t>
   </si>
 </sst>
 </file>
@@ -1668,7 +1671,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -1677,13 +1680,13 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>3</v>
@@ -1692,16 +1695,16 @@
         <v>4</v>
       </c>
       <c r="J1" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="K1" s="4" t="s">
-        <v>232</v>
-      </c>
       <c r="L1" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>5</v>
@@ -1709,41 +1712,41 @@
     </row>
     <row r="2" spans="1:14" ht="57">
       <c r="A2" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>229</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>166</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>181</v>
-      </c>
       <c r="I2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N2" s="3" t="s">
         <v>8</v>
@@ -1751,10 +1754,10 @@
     </row>
     <row r="3" spans="1:14" ht="57">
       <c r="A3" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>9</v>
@@ -1763,7 +1766,7 @@
         <v>159</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>166</v>
@@ -1778,14 +1781,14 @@
         <v>7</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>240</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>8</v>
@@ -1793,10 +1796,10 @@
     </row>
     <row r="4" spans="1:14" ht="42.75">
       <c r="A4" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>12</v>
@@ -1805,7 +1808,7 @@
         <v>13</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>166</v>
@@ -1820,10 +1823,10 @@
         <v>7</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>248</v>
       </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
@@ -1833,43 +1836,43 @@
     </row>
     <row r="5" spans="1:14" ht="42.75">
       <c r="A5" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>8</v>
@@ -1877,10 +1880,10 @@
     </row>
     <row r="6" spans="1:14" ht="57">
       <c r="A6" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>18</v>
@@ -1889,31 +1892,31 @@
         <v>19</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>20</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J6" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>243</v>
-      </c>
       <c r="L6" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>8</v>
@@ -1921,10 +1924,10 @@
     </row>
     <row r="7" spans="1:14" ht="42.75">
       <c r="A7" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>22</v>
@@ -1933,10 +1936,10 @@
         <v>23</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>24</v>
@@ -1948,14 +1951,14 @@
         <v>17</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K7" s="3"/>
       <c r="L7" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N7" s="3" t="s">
         <v>8</v>
@@ -1963,10 +1966,10 @@
     </row>
     <row r="8" spans="1:14" ht="57">
       <c r="A8" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>173</v>
@@ -1975,31 +1978,31 @@
         <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>26</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>8</v>
@@ -2007,19 +2010,19 @@
     </row>
     <row r="9" spans="1:14" ht="128.25">
       <c r="A9" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>167</v>
@@ -2028,22 +2031,22 @@
         <v>169</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>8</v>
@@ -2051,10 +2054,10 @@
     </row>
     <row r="10" spans="1:14" ht="57">
       <c r="A10" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>28</v>
@@ -2063,13 +2066,13 @@
         <v>29</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>176</v>
+        <v>392</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>30</v>
@@ -2079,9 +2082,11 @@
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+      <c r="L10" s="3" t="s">
+        <v>393</v>
+      </c>
       <c r="M10" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>32</v>
@@ -2089,10 +2094,10 @@
     </row>
     <row r="11" spans="1:14" ht="57">
       <c r="A11" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>33</v>
@@ -2101,7 +2106,7 @@
         <v>160</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>167</v>
@@ -2110,20 +2115,20 @@
         <v>161</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="K11" s="3"/>
       <c r="L11" s="3" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>8</v>
@@ -2131,10 +2136,10 @@
     </row>
     <row r="12" spans="1:14" ht="57">
       <c r="A12" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>34</v>
@@ -2143,31 +2148,31 @@
         <v>35</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>8</v>
@@ -2175,10 +2180,10 @@
     </row>
     <row r="13" spans="1:14" ht="57">
       <c r="A13" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>36</v>
@@ -2187,7 +2192,7 @@
         <v>37</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>167</v>
@@ -2196,22 +2201,22 @@
         <v>38</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>8</v>
@@ -2219,10 +2224,10 @@
     </row>
     <row r="14" spans="1:14" ht="57">
       <c r="A14" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>39</v>
@@ -2231,7 +2236,7 @@
         <v>40</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>167</v>
@@ -2240,22 +2245,22 @@
         <v>41</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J14" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="K14" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="K14" s="3" t="s">
-        <v>256</v>
-      </c>
       <c r="L14" s="3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>8</v>
@@ -2263,10 +2268,10 @@
     </row>
     <row r="15" spans="1:14" ht="57">
       <c r="A15" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>42</v>
@@ -2275,31 +2280,31 @@
         <v>43</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G15" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J15" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="H15" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J15" s="3" t="s">
+      <c r="K15" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="K15" s="3" t="s">
-        <v>295</v>
-      </c>
       <c r="L15" s="3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>8</v>
@@ -2307,10 +2312,10 @@
     </row>
     <row r="16" spans="1:14" ht="57">
       <c r="A16" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>45</v>
@@ -2319,31 +2324,31 @@
         <v>46</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G16" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="H16" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>297</v>
-      </c>
       <c r="K16" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>8</v>
@@ -2351,10 +2356,10 @@
     </row>
     <row r="17" spans="1:14" ht="57">
       <c r="A17" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>47</v>
@@ -2363,7 +2368,7 @@
         <v>48</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>167</v>
@@ -2372,20 +2377,20 @@
         <v>49</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>44</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="3" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>8</v>
@@ -2393,10 +2398,10 @@
     </row>
     <row r="18" spans="1:14" ht="57">
       <c r="A18" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>51</v>
@@ -2405,7 +2410,7 @@
         <v>52</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>167</v>
@@ -2414,22 +2419,22 @@
         <v>53</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>8</v>
@@ -2437,10 +2442,10 @@
     </row>
     <row r="19" spans="1:14" ht="57">
       <c r="A19" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>54</v>
@@ -2449,31 +2454,31 @@
         <v>55</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>137</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>8</v>
@@ -2481,10 +2486,10 @@
     </row>
     <row r="20" spans="1:14" ht="85.5">
       <c r="A20" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>56</v>
@@ -2493,7 +2498,7 @@
         <v>57</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>137</v>
@@ -2508,14 +2513,14 @@
         <v>60</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="K20" s="3" t="s">
         <v>336</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>337</v>
       </c>
       <c r="L20" s="3"/>
       <c r="M20" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>50</v>
@@ -2523,10 +2528,10 @@
     </row>
     <row r="21" spans="1:14" ht="42.75">
       <c r="A21" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>61</v>
@@ -2535,13 +2540,13 @@
         <v>62</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>63</v>
@@ -2550,16 +2555,16 @@
         <v>7</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>8</v>
@@ -2567,10 +2572,10 @@
     </row>
     <row r="22" spans="1:14" ht="42.75">
       <c r="A22" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>64</v>
@@ -2579,10 +2584,10 @@
         <v>65</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>66</v>
@@ -2594,16 +2599,16 @@
         <v>7</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>8</v>
@@ -2611,10 +2616,10 @@
     </row>
     <row r="23" spans="1:14" ht="42.75">
       <c r="A23" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>68</v>
@@ -2623,13 +2628,13 @@
         <v>69</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>70</v>
@@ -2638,16 +2643,16 @@
         <v>7</v>
       </c>
       <c r="J23" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="K23" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="K23" s="3" t="s">
-        <v>265</v>
-      </c>
       <c r="L23" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>8</v>
@@ -2655,10 +2660,10 @@
     </row>
     <row r="24" spans="1:14" ht="57">
       <c r="A24" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>71</v>
@@ -2667,13 +2672,13 @@
         <v>170</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>72</v>
@@ -2682,16 +2687,16 @@
         <v>7</v>
       </c>
       <c r="J24" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="K24" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="K24" s="3" t="s">
-        <v>267</v>
-      </c>
       <c r="L24" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>8</v>
@@ -2699,10 +2704,10 @@
     </row>
     <row r="25" spans="1:14" ht="42.75">
       <c r="A25" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>73</v>
@@ -2711,29 +2716,29 @@
         <v>74</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>8</v>
@@ -2741,10 +2746,10 @@
     </row>
     <row r="26" spans="1:14" ht="99.75">
       <c r="A26" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>75</v>
@@ -2753,10 +2758,10 @@
         <v>171</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>76</v>
@@ -2768,16 +2773,16 @@
         <v>78</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N26" s="3" t="s">
         <v>8</v>
@@ -2785,10 +2790,10 @@
     </row>
     <row r="27" spans="1:14" ht="71.25">
       <c r="A27" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>79</v>
@@ -2797,31 +2802,31 @@
         <v>80</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>137</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H27" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="I27" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="I27" s="3" t="s">
-        <v>334</v>
-      </c>
       <c r="J27" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="K27" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="K27" s="3" t="s">
-        <v>271</v>
-      </c>
       <c r="L27" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="N27" s="3" t="s">
         <v>8</v>
@@ -2829,10 +2834,10 @@
     </row>
     <row r="28" spans="1:14" ht="99.75">
       <c r="A28" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>81</v>
@@ -2841,13 +2846,13 @@
         <v>82</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>145</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>83</v>
@@ -2856,16 +2861,16 @@
         <v>162</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>8</v>
@@ -2873,10 +2878,10 @@
     </row>
     <row r="29" spans="1:14" ht="71.25">
       <c r="A29" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>84</v>
@@ -2885,7 +2890,7 @@
         <v>85</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>172</v>
@@ -2900,16 +2905,16 @@
         <v>88</v>
       </c>
       <c r="J29" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="K29" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="K29" s="3" t="s">
-        <v>273</v>
-      </c>
       <c r="L29" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="N29" s="3" t="s">
         <v>8</v>
@@ -2917,28 +2922,28 @@
     </row>
     <row r="30" spans="1:14" ht="42.75">
       <c r="A30" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>163</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>89</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>7</v>
@@ -2947,13 +2952,13 @@
         <v>90</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N30" s="3" t="s">
         <v>8</v>
@@ -2961,43 +2966,43 @@
     </row>
     <row r="31" spans="1:14" ht="42.75">
       <c r="A31" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>91</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>92</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J31" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="K31" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="K31" s="3" t="s">
-        <v>275</v>
-      </c>
       <c r="L31" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="N31" s="3" t="s">
         <v>8</v>
@@ -3005,10 +3010,10 @@
     </row>
     <row r="32" spans="1:14" ht="57">
       <c r="A32" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>93</v>
@@ -3017,7 +3022,7 @@
         <v>94</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>147</v>
@@ -3026,22 +3031,22 @@
         <v>95</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>8</v>
@@ -3049,10 +3054,10 @@
     </row>
     <row r="33" spans="1:14" ht="42.75">
       <c r="A33" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>96</v>
@@ -3061,7 +3066,7 @@
         <v>97</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>147</v>
@@ -3070,22 +3075,22 @@
         <v>98</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N33" s="3" t="s">
         <v>8</v>
@@ -3093,10 +3098,10 @@
     </row>
     <row r="34" spans="1:14" ht="42.75">
       <c r="A34" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>99</v>
@@ -3105,7 +3110,7 @@
         <v>100</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>147</v>
@@ -3114,22 +3119,22 @@
         <v>101</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N34" s="3" t="s">
         <v>8</v>
@@ -3137,10 +3142,10 @@
     </row>
     <row r="35" spans="1:14" ht="57">
       <c r="A35" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>102</v>
@@ -3149,7 +3154,7 @@
         <v>103</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>147</v>
@@ -3158,22 +3163,22 @@
         <v>104</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N35" s="3" t="s">
         <v>8</v>
@@ -3181,10 +3186,10 @@
     </row>
     <row r="36" spans="1:14" ht="71.25">
       <c r="A36" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>105</v>
@@ -3193,29 +3198,29 @@
         <v>106</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N36" s="3" t="s">
         <v>8</v>
@@ -3223,10 +3228,10 @@
     </row>
     <row r="37" spans="1:14" ht="71.25">
       <c r="A37" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>107</v>
@@ -3235,29 +3240,29 @@
         <v>108</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>109</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="3" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N37" s="3" t="s">
         <v>8</v>
@@ -3265,10 +3270,10 @@
     </row>
     <row r="38" spans="1:14" ht="71.25">
       <c r="A38" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>110</v>
@@ -3277,29 +3282,29 @@
         <v>111</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>112</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="3" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N38" s="3" t="s">
         <v>8</v>
@@ -3307,10 +3312,10 @@
     </row>
     <row r="39" spans="1:14" ht="57">
       <c r="A39" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>114</v>
@@ -3319,29 +3324,29 @@
         <v>165</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>164</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N39" s="3" t="s">
         <v>8</v>
@@ -3349,10 +3354,10 @@
     </row>
     <row r="40" spans="1:14" ht="57">
       <c r="A40" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>115</v>
@@ -3361,29 +3366,29 @@
         <v>116</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>117</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>8</v>
@@ -3391,10 +3396,10 @@
     </row>
     <row r="41" spans="1:14" ht="71.25">
       <c r="A41" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>118</v>
@@ -3403,10 +3408,10 @@
         <v>119</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>120</v>
@@ -3427,7 +3432,7 @@
         <v>7</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N41" s="3" t="s">
         <v>8</v>
@@ -3435,10 +3440,10 @@
     </row>
     <row r="42" spans="1:14" ht="85.5">
       <c r="A42" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>121</v>
@@ -3447,29 +3452,29 @@
         <v>122</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>149</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>7</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N42" s="3" t="s">
         <v>8</v>
@@ -3477,10 +3482,10 @@
     </row>
     <row r="43" spans="1:14" ht="85.5">
       <c r="A43" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>123</v>
@@ -3489,7 +3494,7 @@
         <v>124</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>149</v>
@@ -3513,7 +3518,7 @@
         <v>7</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N43" s="3" t="s">
         <v>8</v>
@@ -3521,10 +3526,10 @@
     </row>
     <row r="44" spans="1:14" ht="71.25">
       <c r="A44" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>125</v>
@@ -3533,7 +3538,7 @@
         <v>126</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>168</v>
@@ -3557,10 +3562,10 @@
     </row>
     <row r="45" spans="1:14" ht="57">
       <c r="A45" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>129</v>
@@ -3569,7 +3574,7 @@
         <v>130</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>168</v>
@@ -3593,10 +3598,10 @@
     </row>
     <row r="46" spans="1:14" ht="71.25">
       <c r="A46" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>133</v>
@@ -3605,7 +3610,7 @@
         <v>134</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>168</v>
@@ -3645,10 +3650,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="28.5">
       <c r="A1" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="28.5">
@@ -3656,15 +3661,15 @@
         <v>143</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="28.5">
       <c r="A3" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>310</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -3672,23 +3677,23 @@
         <v>151</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" spans="1:2">

</xml_diff>